<commit_message>
Adele review round 1 + Gus title: 12 fixes across home, approach, footer, BC team, AB team, contact
</commit_message>
<xml_diff>
--- a/MCW VEC Website - Marketing Comments Tracker.xlsx
+++ b/MCW VEC Website - Marketing Comments Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="154">
   <si>
     <t xml:space="preserve">MCW VEC Website — Marketing Team Comments Tracker</t>
   </si>
@@ -394,13 +394,7 @@
     <t xml:space="preserve">Gus is a Principal.</t>
   </si>
   <si>
-    <t xml:space="preserve">Accept and update. Currently listed as 'Senior Electrical / ICAT Lead'. Update to 'Principal'. Note: user previously confirmed the prior title was correct — reconcile internally with Adele before pushing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collin (verify, then web)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Title conflict to resolve</t>
+    <t xml:space="preserve">Done. Updated title from 'Senior Electrical / ICAT Lead' to 'Principal — Electrical / ICAT' — keeps ICAT specialty visible while reflecting Principal status. Bio also updated to lead with 'A Principal at MCW...'</t>
   </si>
   <si>
     <t xml:space="preserve">Missing Calgary Principals</t>
@@ -1281,7 +1275,7 @@
       </c>
       <c r="O6" s="5" t="n">
         <f aca="false">COUNTIF(J5:J34,"Pending")</f>
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1367,7 +1361,7 @@
       </c>
       <c r="O8" s="5" t="n">
         <f aca="false">COUNTIF(J5:J34,"Updated")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2048,17 +2042,17 @@
         <v>123</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>124</v>
+        <v>37</v>
       </c>
       <c r="I27" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="J27" s="8" t="s">
-        <v>26</v>
+      <c r="J27" s="11" t="s">
+        <v>38</v>
       </c>
       <c r="K27" s="7"/>
       <c r="L27" s="7" t="s">
-        <v>125</v>
+        <v>39</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2075,16 +2069,16 @@
         <v>111</v>
       </c>
       <c r="E28" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="G28" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="F28" s="9" t="s">
+      <c r="H28" s="9" t="s">
         <v>127</v>
-      </c>
-      <c r="G28" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="H28" s="9" t="s">
-        <v>129</v>
       </c>
       <c r="I28" s="12" t="s">
         <v>49</v>
@@ -2094,7 +2088,7 @@
       </c>
       <c r="K28" s="9"/>
       <c r="L28" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2111,16 +2105,16 @@
         <v>111</v>
       </c>
       <c r="E29" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="G29" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="H29" s="7" t="s">
         <v>132</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>134</v>
       </c>
       <c r="I29" s="13" t="s">
         <v>31</v>
@@ -2130,7 +2124,7 @@
       </c>
       <c r="K29" s="7"/>
       <c r="L29" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2147,16 +2141,16 @@
         <v>111</v>
       </c>
       <c r="E30" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="G30" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="F30" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="G30" s="9" t="s">
-        <v>138</v>
-      </c>
       <c r="H30" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I30" s="12" t="s">
         <v>49</v>
@@ -2166,7 +2160,7 @@
       </c>
       <c r="K30" s="9"/>
       <c r="L30" s="9" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2180,16 +2174,16 @@
         <v>19</v>
       </c>
       <c r="D31" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="F31" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="E31" s="7" t="s">
+      <c r="G31" s="7" t="s">
         <v>141</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>143</v>
       </c>
       <c r="H31" s="7" t="s">
         <v>37</v>
@@ -2202,7 +2196,7 @@
       </c>
       <c r="K31" s="7"/>
       <c r="L31" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2216,19 +2210,19 @@
         <v>19</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E32" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="G32" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="F32" s="9" t="s">
+      <c r="H32" s="9" t="s">
         <v>146</v>
-      </c>
-      <c r="G32" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>148</v>
       </c>
       <c r="I32" s="8" t="s">
         <v>25</v>
@@ -2238,7 +2232,7 @@
       </c>
       <c r="K32" s="9"/>
       <c r="L32" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2252,16 +2246,16 @@
         <v>19</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E33" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="G33" s="7" t="s">
         <v>150</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="G33" s="7" t="s">
-        <v>152</v>
       </c>
       <c r="H33" s="7" t="s">
         <v>37</v>
@@ -2288,16 +2282,16 @@
         <v>19</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E34" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="G34" s="9" t="s">
         <v>153</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="G34" s="9" t="s">
-        <v>155</v>
       </c>
       <c r="H34" s="9" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
Adele review: 15 fixes — footer bug, geography, wordmark, brand spacing, P3 bridging, PIT, EGBC, Calgary sectors, Vancouver staff count, Gus → Principal, What we'll need layout, Todd LEED simplified
</commit_message>
<xml_diff>
--- a/MCW VEC Website - Marketing Comments Tracker.xlsx
+++ b/MCW VEC Website - Marketing Comments Tracker.xlsx
@@ -2064,7 +2064,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="56" customHeight="1">
+    <row r="29" ht="70" customHeight="1">
       <c r="A29" s="7" t="n">
         <v>25</v>
       </c>
@@ -2095,12 +2095,12 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Discuss. User previously confirmed 'LEED AP (Canada and US)'. Adele questions whether US designation adds value for BC/AB clients. Recommend simplifying to 'LEED AP' unless Todd specifically wants to keep both.</t>
+          <t>Done. Simplified to 'P.Eng. · LEED AP · Edmonton' on the AB Team card; bio updated to 'A LEED Accredited Professional' (was 'in both Canada and the US'). Contact page already said 'LEED AP' — no change there. If Todd wants the US designation reinstated, easy to revert.</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>Collin to confirm with Todd</t>
+          <t>Collin (web)</t>
         </is>
       </c>
       <c r="I29" s="13" t="inlineStr">
@@ -2108,15 +2108,15 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="J29" s="11" t="inlineStr">
+        <is>
+          <t>Updated</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr"/>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>Cosmetic</t>
+          <t>Live after next push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace Canada map with Adele's new image (pins baked in); Todd LEED simplified
</commit_message>
<xml_diff>
--- a/MCW VEC Website - Marketing Comments Tracker.xlsx
+++ b/MCW VEC Website - Marketing Comments Tracker.xlsx
@@ -2232,7 +2232,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="40" customHeight="1">
+    <row r="32" ht="84" customHeight="1">
       <c r="A32" s="9" t="n">
         <v>28</v>
       </c>
@@ -2263,12 +2263,12 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>Defer until Adele sends the new map. Current Canada map is the user-supplied PNG with city dots overlaid.</t>
+          <t>Done. Adele's new map (Map/Map.jpg, 863x760 — Canada outline with green pins already placed at all MCW office cities) installed as assets/canada-map.jpg. Replaced the previous SVG+overlay-dots structure with a single clean img element. Map legend kept beneath. CSS unchanged (canada-map container already styles correctly).</t>
         </is>
       </c>
       <c r="H32" s="9" t="inlineStr">
         <is>
-          <t>Adele to send</t>
+          <t>Collin (web)</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr">
@@ -2276,15 +2276,15 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="J32" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="J32" s="11" t="inlineStr">
+        <is>
+          <t>Updated</t>
         </is>
       </c>
       <c r="K32" s="9" t="inlineStr"/>
       <c r="L32" s="9" t="inlineStr">
         <is>
-          <t>Waiting on Adele</t>
+          <t>Live after next push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Page titles aligned to new wordmark (MCW VEC → MCW Collaborative Delivery)
</commit_message>
<xml_diff>
--- a/MCW VEC Website - Marketing Comments Tracker.xlsx
+++ b/MCW VEC Website - Marketing Comments Tracker.xlsx
@@ -870,7 +870,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="98" customHeight="1">
+    <row r="8" ht="112" customHeight="1">
       <c r="A8" s="9" t="n">
         <v>4</v>
       </c>
@@ -901,7 +901,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Done. Adopted Adele's version. Top line now reads 'Collaborative Delivery' and bottom line 'from Vancouver • Edmonton • Calgary' (uppercase + tracked). Mobile sub-line font reduced (0.62rem → 0.55rem, letter-spacing 0.08em → 0.04em) to fit longer text on phones. CSS cache bumped to v=15. Note: page titles in browser tabs still say 'MCW VEC' — let me know if you want those updated too.</t>
+          <t>Done. Adopted Adele's version. Top line now reads 'Collaborative Delivery' and bottom line 'from Vancouver • Edmonton • Calgary' (uppercase + tracked). Mobile sub-line font reduced (0.62rem → 0.55rem, letter-spacing 0.08em → 0.04em) to fit longer text on phones. CSS cache bumped to v=15. Browser-tab page titles also updated to drop 'MCW VEC' — now use 'MCW Collaborative Delivery' across all 37 pages.</t>
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Remove Cowichan Tribes Status reference from James Furlong profile pending consent
</commit_message>
<xml_diff>
--- a/MCW VEC Website - Marketing Comments Tracker.xlsx
+++ b/MCW VEC Website - Marketing Comments Tracker.xlsx
@@ -1840,7 +1840,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="42" customHeight="1">
+    <row r="25" ht="70" customHeight="1">
       <c r="A25" s="7" t="n">
         <v>21</v>
       </c>
@@ -1871,12 +1871,12 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Action required. Collin to confirm with James Furlong before this site is shared with anyone external. Until confirmed, consider removing 'Cowichan Tribes' from his credentials line.</t>
+          <t>Done. Removed 'Cowichan Tribes' from credentials line (now 'MBA · CET · CEM · LEED AP · Calgary') and removed the 'He is a status indigenous person of the Cowichan Tribes' sentence from his bio. James can request reinstatement once he gives explicit consent.</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>Collin to confirm with James</t>
+          <t>Collin (web)</t>
         </is>
       </c>
       <c r="I25" s="12" t="inlineStr">
@@ -1884,15 +1884,15 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J25" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="J25" s="11" t="inlineStr">
+        <is>
+          <t>Updated</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr"/>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>Compliance / consent</t>
+          <t>Live after next push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Alliance contracts to home page collaborative-delivery list (forward-looking framing)
</commit_message>
<xml_diff>
--- a/MCW VEC Website - Marketing Comments Tracker.xlsx
+++ b/MCW VEC Website - Marketing Comments Tracker.xlsx
@@ -1056,7 +1056,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
+    <row r="11" ht="84" customHeight="1">
       <c r="A11" s="7" t="n">
         <v>7</v>
       </c>
@@ -1087,12 +1087,12 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Discuss. Alliance contracting (true alliancing, not just IPD) is gaining traction in BC infrastructure. Recommend adding once MCW has a confirmed Alliance reference, otherwise list as 'in pursuit'.</t>
+          <t>Done. Added Alliance to the home page 'Why MCW for Collaborative Delivery' lede with explicit forward-looking framing: 'IPD, CMAR, P3, Progressive Design-Build, and Alliance contracts as they emerge in Canadian infrastructure procurement.' Signals readiness without claiming project experience MCW does not yet have.</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>Collin / Adele</t>
+          <t>Collin</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
@@ -1100,15 +1100,15 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="J11" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>Updated</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr"/>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>Need leadership input</t>
+          <t>Live after next push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Graham Lovely IPD experience (TOL Fire Hall 5, Kamloops Arts Centre) to BC Team bio
</commit_message>
<xml_diff>
--- a/MCW VEC Website - Marketing Comments Tracker.xlsx
+++ b/MCW VEC Website - Marketing Comments Tracker.xlsx
@@ -1504,7 +1504,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="40" customHeight="1">
+    <row r="19" ht="70" customHeight="1">
       <c r="A19" s="7" t="n">
         <v>15</v>
       </c>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Accept. Update Graham's bc-team.html bio to call out specific IPD project work and his role under collaborative delivery agreements.</t>
+          <t>Done. Added to Graham's bio: 'IPD experience includes the Township of Langley Fire Hall No. 5 and Training Centre, and the Kamloops Centre for the Arts — leading electrical scope within integrated project teams.' (Both projects are featured on the Experience page.)</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -1548,15 +1548,15 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="J19" s="11" t="inlineStr">
+        <is>
+          <t>Updated</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr"/>
       <c r="L19" s="7" t="inlineStr">
         <is>
-          <t>Need IPD project list from Graham</t>
+          <t>Live after next push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BC Team expanded: Josh Tanner added to Associates + new Project Managers section (15 new cards with headshots, bios, and credentials from Master Resume List)
</commit_message>
<xml_diff>
--- a/MCW VEC Website - Marketing Comments Tracker.xlsx
+++ b/MCW VEC Website - Marketing Comments Tracker.xlsx
@@ -1616,7 +1616,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="56" customHeight="1">
+    <row r="21" ht="126" customHeight="1">
       <c r="A21" s="7" t="n">
         <v>17</v>
       </c>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Accept. Restructure BC Team page: replace 'Associates' grouping with 'Project Managers' umbrella, which lets us include Kaan (KCA project) alongside Melissa and Matt. Add Josh Tanner to the same group (per next comment).</t>
+          <t>Done. Added new 'Project Managers and engineering staff' section under the existing Associates section. 15 new cards populated (Sean Farrell, Lucy Kryachok, Hussam Iskander, Blake Steptoe, Evan Lok, Jonathan Lau, Kaan Ertan, Scott MacLaren, Huy Nguyen, Rick Arikado, Alan Jones, Benjamin Ellah, Laura Muñoz, Lloyd Yodogawa, Steve Nixon) with bios extracted from the Master Resume List and face-aware-cropped headshots. Kaan's bio references the Kamloops Centre for the Arts project.</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -1660,19 +1660,19 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="J21" s="11" t="inlineStr">
+        <is>
+          <t>Updated</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr"/>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>Need PM list + bios + headshots</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="40" customHeight="1">
+          <t>Live after next push</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="56" customHeight="1">
       <c r="A22" s="9" t="n">
         <v>18</v>
       </c>
@@ -1703,12 +1703,12 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Accept. Add Josh Tanner to BC Team under PM/Associate group. Need bio + headshot.</t>
+          <t>Done. Added Josh Tanner as third Associate (Associate — Electrical, P.Eng. BC, B.Eng. UVic). Bio reflects 9 years prior experience + electrical engineering, lighting design and controls, power distribution, PV, EV specialties.</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
-          <t>Collin to source content</t>
+          <t>Collin (web)</t>
         </is>
       </c>
       <c r="I22" s="12" t="inlineStr">
@@ -1716,15 +1716,15 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J22" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="J22" s="11" t="inlineStr">
+        <is>
+          <t>Updated</t>
         </is>
       </c>
       <c r="K22" s="9" t="inlineStr"/>
       <c r="L22" s="9" t="inlineStr">
         <is>
-          <t>Need bio + headshot</t>
+          <t>Live after next push</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>Accept. Resolved by 'Add Josh Tanner' action above. Once Josh is added, count goes from 2 to 3.</t>
+          <t>Done. Associates section now shows 3 cards: Melissa Smith, Matt Clayton, Josh Tanner.</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr">
@@ -1828,15 +1828,15 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="J24" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>Updated</t>
         </is>
       </c>
       <c r="K24" s="9" t="inlineStr"/>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Bundled with Josh add</t>
+          <t>Live after next push</t>
         </is>
       </c>
     </row>

</xml_diff>